<commit_message>
aicore: /aicore/lisanslama sayfası + modül fiyat modeli ayrımı
Site:
- Yeni sayfa /aicore/lisanslama — müşteriye dönük yapay zekâ lisanslama
  anlatımı: iki kullanım şekli, ücretlendirilmeyenler, sayaç neyi sayar
  (bitmiş iş + 1/2/5 ağırlık), sürpriz fatura yok (%70/85/95/100), şeffaflık,
  6 soruluk SSS

Görev Paneli:
- Altyapı exceli: Fiyat modeli + gerekçe sütunu (32 modül), Fiyat Modeli
  özet sayfası, GateCoreAI satırı
- Backend iş paketi v4: bitmiş-iş sayacı, kayıt açan trafik muafiyeti,
  üç lisans ürünü, sessiz ölçüm + pilot adımı
- Yeni: iş modeli ders anlatımı, yönetici karar sayfası (8 karar), sunum
</commit_message>
<xml_diff>
--- a/gorevler/ekler/aicore-altyapi-gereksinimleri/AICore_Altyapi_Gereksinimleri.xlsx
+++ b/gorevler/ekler/aicore-altyapi-gereksinimleri/AICore_Altyapi_Gereksinimleri.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kademeler" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ortak Gereksinimler" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eklenti Notları" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notlar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiyat Modeli" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eklenti Notları" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notlar" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +36,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +51,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004C1D95"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F0FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -70,6 +85,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -847,7 +874,205 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>AICore eklentileri — fiyat modeli ayrımı</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>KURAL</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kişi başına: teknisyen (veya yönetici) ekranda; o kişi olmadan eklenti çalışmaz; değer kişi sayısıyla artar. → lisansa yıllık sabit ek ücret.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Sabit: kayıt, varlık, doküman veya son kullanıcı hacmiyle çalışır; kimin giriş yaptığından bağımsız. → kurum başına yıllık sabit bedel, hacim bandına göre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>KİŞİ BAŞINA (7)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>SolveCoreAI · ReplyCoreAI · ToneCoreAI · VoiceCoreAI · CallCoreAI · CoachCoreAI · ReportCoreAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ReportCoreAI teknisyen değil YÖNETİCİ koltuğuna bağlanır (rapor kullanan kişi sayısı).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>SABİT (24)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>KnowCoreAI · DocCoreAI · RootCoreAI · MergeCoreAI · ChatCoreAI · ClassifyCoreAI · PriorityCoreAI · ImpactCoreAI · PredictCoreAI · SentimentCoreAI · KBCoreAI · StormCoreAI · FlowCoreAI · DisCoreAI · TranslateCoreAI · VisionCoreAI · ShiftCoreAI · AuditCoreAI · AssetCoreAI · VendorCoreAI · ContractCoreAI · BudgetCoreAI · ProjectCoreAI · RisiCoreAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Sabit fiyatın bandı her eklentinin kendi ölçüsüne göre belirlenir (kayıt hacmi, varlık sayısı, çalışan sayısı...). Ölçü sütunu: "Boyutlandırma etkeni".</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>KARAR BEKLEYEN 5</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Aşağıdakiler iki modele de oturuyor; ticari tercih gerekiyor:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>ToneCoreAI</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Teknisyen yanıt yazarken çalışır (kişi başına) — ama ölçüsü yanıt hacmi (sabit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>CallCoreAI</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Çağrı merkezi teknisyeninin işini alır (kişi başına) — ama ölçüsü çağrı hacmi (sabit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>VoiceCoreAI</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Saha teknisyeni kullanıyorsa kişi başına; son kullanıcıya telefon kanalı açılırsa sabit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>TranslateCoreAI</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Yalnız teknisyen tarafında kullanılırsa kişi başına; iki tarafta da mesaja giriyorsa sabit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>ImpactCoreAI</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Değişiklik kaydına bağlı (sabit) — ama değişiklik yöneticisi koltuğuna da bağlanabilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>NOT</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>GateCoreAI bu sayfada yok: eklenti değil, kurumun kendi yapay zekâsının bağlandığı kapı. Kurum başına sabit + insansız biten iş için yıllık iş paketi ile fiyatlanır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Kaynak model: aicore/Yonetici_Ozeti_ve_Kararlar.md (25.07.2026). Sabit bedellerin rakamı sessiz ölçüm sonrası netleşir.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -855,6 +1080,8 @@
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -883,6 +1110,16 @@
           <t>Boyutlandırma etkeni</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fiyat modeli</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Gerekçe (fiyat modeli)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -910,6 +1147,16 @@
           <t>Teknisyen sayısı + günlük kayıt</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Kişi başına</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Teknisyen kendi ekranında tetikler; onsuz çalışmaz. Değer teknisyen sayısıyla artar.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -937,6 +1184,16 @@
           <t>Kayıt arşivi büyüklüğü</t>
         </is>
       </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Gece toplu çalışır, ortada teknisyen yok. Yük kayıt arşiviyle ölçeklenir.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -964,6 +1221,16 @@
           <t>Doküman hacmi</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Doküman hacmiyle çalışır; teknisyen sayısından bağımsız.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -991,6 +1258,16 @@
           <t>Geri bildirim hacmi</t>
         </is>
       </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Gece toplu; geri bildirim hacmiyle ölçeklenir.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1018,6 +1295,16 @@
           <t>Günlük kayıt hacmi</t>
         </is>
       </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Yeni kayıt geldiğinde sistem tetikler, teknisyen değil. Kayıt hacmine bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1045,6 +1332,16 @@
           <t>TOPLAM ÇALIŞAN sayısı + eşzamanlı sohbet</t>
         </is>
       </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Son kullanıcıya hizmet eder; ölçü TOPLAM ÇALIŞAN sayısı. Çalışan bandına göre sabit fiyat.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1072,6 +1369,16 @@
           <t>Teknisyen sayısı + günlük kayıt</t>
         </is>
       </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Kişi başına</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Teknisyenin yanıt taslağını hazırlar; gönderim teknisyende. Teknisyen sayısıyla ölçeklenir.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1099,6 +1406,16 @@
           <t>Günlük kayıt hacmi</t>
         </is>
       </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Her yeni kayıtta otomatik çalışır; insansız. Kayıt hacmine bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1126,6 +1443,16 @@
           <t>Günlük kayıt hacmi</t>
         </is>
       </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Her yeni kayıtta otomatik; insansız. Kayıt hacmine bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1153,6 +1480,16 @@
           <t>Aylık değişiklik sayısı</t>
         </is>
       </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Değişiklik kaydı başına çalışır; ölçü aylık değişiklik sayısı. (Sınırda: değişiklik yöneticisi koltuğuna da bağlanabilir.)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1180,6 +1517,16 @@
           <t>Kayıt hacmi</t>
         </is>
       </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik analiz; insansız. Kayıt hacmine bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1207,6 +1554,16 @@
           <t>Rapor kullanan yönetici sayısı</t>
         </is>
       </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Kişi başına</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Soruyu bir insan sorar; ölçü rapor kullanan yönetici sayısı. NOT: teknisyen değil, YÖNETİCİ koltuğu.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1234,6 +1591,16 @@
           <t>Günlük mesaj hacmi</t>
         </is>
       </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Mesajlar üzerinde otomatik; insansız. Mesaj hacmine bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1261,6 +1628,16 @@
           <t>Bilgi bankası büyüklüğü</t>
         </is>
       </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Bilgi bankası üzerinde toplu çalışır; teknisyen sayısından bağımsız.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1288,6 +1665,16 @@
           <t>Günlük yanıt hacmi</t>
         </is>
       </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Kişi başına</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Teknisyen yanıt yazarken çalışır, o oturuma bağlı. (Sınırda: yanıt hacmiyle sabit de fiyatlanabilir.)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1315,6 +1702,16 @@
           <t>Alarm/olay tepe hacmi</t>
         </is>
       </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Alarm akışında otomatik; insansız. Tepe olay hacmine bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1342,6 +1739,16 @@
           <t>Düşük — hacimden bağımsız</t>
         </is>
       </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Yönetici ara sıra kullanır, hacimden bağımsız. Kurum başına sabit.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1369,6 +1776,16 @@
           <t>Varlık sayısı</t>
         </is>
       </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik ağ taraması; insansız. Varlık sayısına bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1396,6 +1813,16 @@
           <t>Çok dilli mesaj hacmi</t>
         </is>
       </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Hem kullanıcı hem teknisyen tarafında mesaj üzerinde çalışır; ölçü mesaj hacmi. (Sınırda: yalnız teknisyen tarafında kullanılırsa kişi başına.)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1423,6 +1850,16 @@
           <t>Günlük çağrı hacmi</t>
         </is>
       </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Kişi başına</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Saha teknisyeni sesle işlem yapar; kişiye bağlı kullanım. (Sınırda: son kullanıcı telefon kanalı açılırsa sabit.)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1450,6 +1887,16 @@
           <t>Günlük çağrı hacmi + kayıt saklama süresi</t>
         </is>
       </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Kişi başına</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Çağrı merkezi teknisyeninin not yükünü alır; koltuğa bağlı. (Sınırda: çağrı hacmiyle sabit de fiyatlanabilir.)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1477,6 +1924,16 @@
           <t>Görsel ekli kayıt oranı</t>
         </is>
       </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Kayıt ekindeki görselde otomatik çalışır; insansız. Görselli kayıt oranına bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1504,6 +1961,16 @@
           <t>Ekip büyüklüğü</t>
         </is>
       </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Tek yönetici tüm ekip için kullanır; ölçü ekip büyüklüğü. Kurum başına sabit, ekip bandıyla.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1531,6 +1998,16 @@
           <t>Süreç/kayıt hacmi</t>
         </is>
       </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik denetim; insansız. Süreç/kayıt hacmine bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1558,6 +2035,16 @@
           <t>Varlık sayısı</t>
         </is>
       </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik; varlık sayısına bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1585,6 +2072,16 @@
           <t>Tedarikçi sayısı</t>
         </is>
       </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik; tedarikçi sayısına bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1612,6 +2109,16 @@
           <t>Sözleşme sayısı</t>
         </is>
       </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Sözleşme deposu üzerinde toplu; sözleşme sayısına bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1639,6 +2146,16 @@
           <t>Kalem sayısı — düşük yük</t>
         </is>
       </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik; kalem sayısına bağlı, yük düşük.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1666,6 +2183,16 @@
           <t>Teknisyen sayısı</t>
         </is>
       </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Kişi başına</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Her teknisyenin performansını ayrı analiz eder; değer doğrudan teknisyen sayısıyla artar.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1693,6 +2220,16 @@
           <t>Aktif proje sayısı</t>
         </is>
       </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik; aktif proje sayısına bağlı.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1718,6 +2255,16 @@
       <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Varlık sayısı</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Periyodik; varlık sayısına bağlı.</t>
         </is>
       </c>
     </row>
@@ -1726,7 +2273,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
aicore: paketleme düzeltmesi — çift ücret kaldırıldı
Erman'ın itirazı: "7 ürün teknisyen bazlı, diğerleri fix price dedim
geçtim; burada başarılı iş başına ayrıca para alıyoruz gibi duruyor."
Haklıydı — modül lisansının üstüne iş sayacı binmiş görünüyordu.

Kural netleşti: lisansı olan iş sayılmaz, lisansı olmayan iş banda girer.

- /aicore/lisanslama baştan yazıldı: teklifte üç kalem (eklentiler ·
  GateCoreAI · kurulum-destek), "eklentinin yaptığı iş fiyatına dahildir"
  bölümü, sayaç ne değildir / ne işe yarar ayrımı, bant yalnız dış ajan için
- Lisanslama rehberi 13. bölüm: iki kural maddesi eklendi
- Ders, karar sayfası, backend yol haritası, altyapı exceli aynı kurala
  hizalandı
- Backend gereksinimi: işi yapan yazılımın eklenti lisansı varsa iş sayılır
  ve raporlanır ama bant havuzundan düşmez

Dayanak: Microsoft (lisanslı kullanıcı arkasındaysa tüketim dahil) ·
ServiceNow'un modül üstüne havuz koyup aldığı yenileme tepkisi ·
SAP/Workday'in dış ajanı kapıdan ölçmesi.
</commit_message>
<xml_diff>
--- a/gorevler/ekler/aicore-altyapi-gereksinimleri/AICore_Altyapi_Gereksinimleri.xlsx
+++ b/gorevler/ekler/aicore-altyapi-gereksinimleri/AICore_Altyapi_Gereksinimleri.xlsx
@@ -874,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -944,12 +944,12 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>SABİT (24)</t>
+          <t>SABİT (25)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>KnowCoreAI · DocCoreAI · RootCoreAI · MergeCoreAI · ChatCoreAI · ClassifyCoreAI · PriorityCoreAI · ImpactCoreAI · PredictCoreAI · SentimentCoreAI · KBCoreAI · StormCoreAI · FlowCoreAI · DisCoreAI · TranslateCoreAI · VisionCoreAI · ShiftCoreAI · AuditCoreAI · AssetCoreAI · VendorCoreAI · ContractCoreAI · BudgetCoreAI · ProjectCoreAI · RisiCoreAI</t>
+          <t>KnowCoreAI · DocCoreAI · RootCoreAI · MergeCoreAI · ChatCoreAI · ClassifyCoreAI · PriorityCoreAI · ImpactCoreAI · PredictCoreAI · SentimentCoreAI · KBCoreAI · StormCoreAI · FlowCoreAI · DisCoreAI · TranslateCoreAI · VisionCoreAI · ShiftCoreAI · AuditCoreAI · AssetCoreAI · VendorCoreAI · ContractCoreAI · BudgetCoreAI · ProjectCoreAI · RisiCoreAI · GateCoreAI</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>GateCoreAI bu sayfada yok: eklenti değil, kurumun kendi yapay zekâsının bağlandığı kapı. Kurum başına sabit + insansız biten iş için yıllık iş paketi ile fiyatlanır.</t>
+          <t>GateCoreAI listeye eklendi (25.07): eklenti değil, kurumun kendi yapay zekâsının bağlandığı kapı. Kurum başına sabit; insansız biten iş ayrıca yıllık iş paketinden düşer.</t>
         </is>
       </c>
     </row>
@@ -1058,6 +1058,41 @@
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Kaynak model: aicore/Yonetici_Ozeti_ve_Kararlar.md (25.07.2026). Sabit bedellerin rakamı sessiz ölçüm sonrası netleşir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>PAKETLEME KURALI</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Teklifte üç kalem vardır: (1) eklentiler — kişi başına ya da sabit, (2) GateCoreAI — zorunlu, kurum başına sabit, (3) kurulum + destek. Dördüncü kalem yoktur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Eklentinin insansız çalışması eklentinin fiyatına DAHİLDİR; iş başına ayrıca ücret alınmaz. Aynı iş iki kez ücretlendirilmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>İş sayacı bir fatura kalemi değildir. İki işi vardır: müşterinin DIŞARIDAN bağladığı ajanların GateCoreAI bandını belirlemek ve kimliğini bildirmeyen otomasyonu yakalamak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Kural tek cümle: lisansı olan iş sayılmaz, lisansı olmayan iş banda girer.</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2265,6 +2300,43 @@
       <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Periyodik; varlık sayısına bağlı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>GateCoreAI</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Yazmaz — kapıdır. Bağlanan yazılımın yetkisi neyse onu uygular; her isteği kimlik ve sorumluyla kaydeder.</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Kurumun kendi yapay zekâsı / dış eklentiler; kimlik ve yetki altyapısı (ServiceCore backend)</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Sürekli — her istekte</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Bağlanan yazılım sayısı + istek hacmi</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Sabit</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Eklenti değil, kurumun kendi yapay zekâsının bağlandığı kapı. Teknisyen sayısıyla ölçeklenmez; kurum başına yıllık sabit bedelle satılır. İnsansız biten iş ayrıca yıllık iş paketinden düşer.</t>
         </is>
       </c>
     </row>

</xml_diff>